<commit_message>
Modules dependency has been generated and other columns have been introduced in reports
</commit_message>
<xml_diff>
--- a/wwwroot/119/BoxBreaking.xlsx
+++ b/wwwroot/119/BoxBreaking.xlsx
@@ -9784,7 +9784,7 @@
         <v>0.1</v>
       </c>
       <c r="J155" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K155" s="0">
         <v>1</v>
@@ -9843,7 +9843,7 @@
         <v>0.1</v>
       </c>
       <c r="J156" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K156" s="0">
         <v>1</v>
@@ -9902,7 +9902,7 @@
         <v>0.1</v>
       </c>
       <c r="J157" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K157" s="0">
         <v>1</v>
@@ -9961,7 +9961,7 @@
         <v>0.1</v>
       </c>
       <c r="J158" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K158" s="0">
         <v>1</v>
@@ -10020,7 +10020,7 @@
         <v>0.1</v>
       </c>
       <c r="J159" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K159" s="0">
         <v>1</v>
@@ -10079,7 +10079,7 @@
         <v>0.1</v>
       </c>
       <c r="J160" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K160" s="0">
         <v>1</v>
@@ -10138,7 +10138,7 @@
         <v>0.1</v>
       </c>
       <c r="J161" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K161" s="0">
         <v>1</v>
@@ -10197,7 +10197,7 @@
         <v>0.1</v>
       </c>
       <c r="J162" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K162" s="0">
         <v>1</v>
@@ -10256,7 +10256,7 @@
         <v>0.1</v>
       </c>
       <c r="J163" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K163" s="0">
         <v>1</v>
@@ -10315,7 +10315,7 @@
         <v>0.1</v>
       </c>
       <c r="J164" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K164" s="0">
         <v>1</v>
@@ -10374,7 +10374,7 @@
         <v>0.1</v>
       </c>
       <c r="J165" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K165" s="0">
         <v>1</v>
@@ -10433,7 +10433,7 @@
         <v>0.1</v>
       </c>
       <c r="J166" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K166" s="0">
         <v>1</v>
@@ -10492,7 +10492,7 @@
         <v>0.1</v>
       </c>
       <c r="J167" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K167" s="0">
         <v>1</v>
@@ -10551,7 +10551,7 @@
         <v>0.1</v>
       </c>
       <c r="J168" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K168" s="0">
         <v>1</v>
@@ -10610,7 +10610,7 @@
         <v>0.1</v>
       </c>
       <c r="J169" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K169" s="0">
         <v>1</v>
@@ -10669,7 +10669,7 @@
         <v>0.1</v>
       </c>
       <c r="J170" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K170" s="0">
         <v>1</v>
@@ -10728,7 +10728,7 @@
         <v>0.1</v>
       </c>
       <c r="J171" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K171" s="0">
         <v>1</v>
@@ -10787,7 +10787,7 @@
         <v>0.1</v>
       </c>
       <c r="J172" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K172" s="0">
         <v>1</v>
@@ -10846,7 +10846,7 @@
         <v>0.1</v>
       </c>
       <c r="J173" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K173" s="0">
         <v>1</v>
@@ -10905,7 +10905,7 @@
         <v>0.1</v>
       </c>
       <c r="J174" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K174" s="0">
         <v>1</v>
@@ -10964,7 +10964,7 @@
         <v>0.1</v>
       </c>
       <c r="J175" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K175" s="0">
         <v>1</v>
@@ -11023,7 +11023,7 @@
         <v>0.1</v>
       </c>
       <c r="J176" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K176" s="0">
         <v>3</v>
@@ -11082,7 +11082,7 @@
         <v>0.1</v>
       </c>
       <c r="J177" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K177" s="0">
         <v>3</v>
@@ -11141,7 +11141,7 @@
         <v>0.1</v>
       </c>
       <c r="J178" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K178" s="0">
         <v>1</v>
@@ -11200,7 +11200,7 @@
         <v>0.1</v>
       </c>
       <c r="J179" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K179" s="0">
         <v>1</v>
@@ -11259,7 +11259,7 @@
         <v>0.1</v>
       </c>
       <c r="J180" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K180" s="0">
         <v>1</v>
@@ -11318,7 +11318,7 @@
         <v>0.1</v>
       </c>
       <c r="J181" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K181" s="0">
         <v>1</v>
@@ -11377,7 +11377,7 @@
         <v>0.1</v>
       </c>
       <c r="J182" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K182" s="0">
         <v>1</v>
@@ -11436,7 +11436,7 @@
         <v>0.1</v>
       </c>
       <c r="J183" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K183" s="0">
         <v>1</v>
@@ -11495,7 +11495,7 @@
         <v>0.1</v>
       </c>
       <c r="J184" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K184" s="0">
         <v>3</v>
@@ -11554,7 +11554,7 @@
         <v>0.1</v>
       </c>
       <c r="J185" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K185" s="0">
         <v>3</v>
@@ -11613,7 +11613,7 @@
         <v>0.1</v>
       </c>
       <c r="J186" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K186" s="0">
         <v>3</v>
@@ -11672,7 +11672,7 @@
         <v>0.1</v>
       </c>
       <c r="J187" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K187" s="0">
         <v>3</v>
@@ -11731,7 +11731,7 @@
         <v>0.1</v>
       </c>
       <c r="J188" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K188" s="0">
         <v>3</v>
@@ -11790,7 +11790,7 @@
         <v>0.1</v>
       </c>
       <c r="J189" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K189" s="0">
         <v>3</v>
@@ -11849,7 +11849,7 @@
         <v>0.1</v>
       </c>
       <c r="J190" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K190" s="0">
         <v>3</v>
@@ -11908,7 +11908,7 @@
         <v>0.1</v>
       </c>
       <c r="J191" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K191" s="0">
         <v>3</v>
@@ -11967,7 +11967,7 @@
         <v>0.1</v>
       </c>
       <c r="J192" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K192" s="0">
         <v>3</v>
@@ -12026,7 +12026,7 @@
         <v>0.1</v>
       </c>
       <c r="J193" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K193" s="0">
         <v>3</v>
@@ -12085,7 +12085,7 @@
         <v>0.1</v>
       </c>
       <c r="J194" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K194" s="0">
         <v>3</v>
@@ -12144,7 +12144,7 @@
         <v>0.1</v>
       </c>
       <c r="J195" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K195" s="0">
         <v>3</v>
@@ -12203,7 +12203,7 @@
         <v>0.1</v>
       </c>
       <c r="J196" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K196" s="0">
         <v>3</v>
@@ -12262,7 +12262,7 @@
         <v>0.1</v>
       </c>
       <c r="J197" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K197" s="0">
         <v>3</v>
@@ -12321,7 +12321,7 @@
         <v>0.1</v>
       </c>
       <c r="J198" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K198" s="0">
         <v>3</v>
@@ -12380,7 +12380,7 @@
         <v>0.1</v>
       </c>
       <c r="J199" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K199" s="0">
         <v>3</v>
@@ -12439,7 +12439,7 @@
         <v>0.1</v>
       </c>
       <c r="J200" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K200" s="0">
         <v>3</v>
@@ -12498,7 +12498,7 @@
         <v>0.1</v>
       </c>
       <c r="J201" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K201" s="0">
         <v>3</v>
@@ -12557,7 +12557,7 @@
         <v>0.1</v>
       </c>
       <c r="J202" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K202" s="0">
         <v>3</v>
@@ -12616,7 +12616,7 @@
         <v>0.1</v>
       </c>
       <c r="J203" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K203" s="0">
         <v>3</v>
@@ -12675,7 +12675,7 @@
         <v>0.1</v>
       </c>
       <c r="J204" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K204" s="0">
         <v>3</v>
@@ -12734,7 +12734,7 @@
         <v>0.1</v>
       </c>
       <c r="J205" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K205" s="0">
         <v>3</v>
@@ -12793,7 +12793,7 @@
         <v>0.1</v>
       </c>
       <c r="J206" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K206" s="0">
         <v>3</v>
@@ -12852,7 +12852,7 @@
         <v>0.1</v>
       </c>
       <c r="J207" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K207" s="0">
         <v>1</v>
@@ -12911,7 +12911,7 @@
         <v>0.1</v>
       </c>
       <c r="J208" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K208" s="0">
         <v>1</v>
@@ -12970,7 +12970,7 @@
         <v>0.1</v>
       </c>
       <c r="J209" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K209" s="0">
         <v>3</v>
@@ -13029,7 +13029,7 @@
         <v>0.1</v>
       </c>
       <c r="J210" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K210" s="0">
         <v>3</v>
@@ -13088,7 +13088,7 @@
         <v>0.1</v>
       </c>
       <c r="J211" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K211" s="0">
         <v>3</v>
@@ -13147,7 +13147,7 @@
         <v>0.1</v>
       </c>
       <c r="J212" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K212" s="0">
         <v>999</v>
@@ -13206,7 +13206,7 @@
         <v>0.1</v>
       </c>
       <c r="J213" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K213" s="0">
         <v>999</v>
@@ -13265,7 +13265,7 @@
         <v>0.1</v>
       </c>
       <c r="J214" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K214" s="0">
         <v>999</v>
@@ -13324,7 +13324,7 @@
         <v>0.1</v>
       </c>
       <c r="J215" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K215" s="0">
         <v>999</v>
@@ -13383,7 +13383,7 @@
         <v>0.1</v>
       </c>
       <c r="J216" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K216" s="0">
         <v>999</v>
@@ -13442,7 +13442,7 @@
         <v>0.1</v>
       </c>
       <c r="J217" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K217" s="0">
         <v>3</v>
@@ -13501,7 +13501,7 @@
         <v>0.1</v>
       </c>
       <c r="J218" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K218" s="0">
         <v>1</v>
@@ -13560,7 +13560,7 @@
         <v>0.1</v>
       </c>
       <c r="J219" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K219" s="0">
         <v>1</v>
@@ -13619,7 +13619,7 @@
         <v>0.1</v>
       </c>
       <c r="J220" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K220" s="0">
         <v>1</v>
@@ -13678,7 +13678,7 @@
         <v>0.1</v>
       </c>
       <c r="J221" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K221" s="0">
         <v>1</v>
@@ -13737,7 +13737,7 @@
         <v>0.1</v>
       </c>
       <c r="J222" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K222" s="0">
         <v>1</v>
@@ -13796,7 +13796,7 @@
         <v>0.1</v>
       </c>
       <c r="J223" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K223" s="0">
         <v>1</v>
@@ -13855,7 +13855,7 @@
         <v>0.1</v>
       </c>
       <c r="J224" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K224" s="0">
         <v>2</v>
@@ -13914,7 +13914,7 @@
         <v>0.1</v>
       </c>
       <c r="J225" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K225" s="0">
         <v>2</v>
@@ -13973,7 +13973,7 @@
         <v>0.1</v>
       </c>
       <c r="J226" s="0" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="K226" s="0">
         <v>2</v>

</xml_diff>